<commit_message>
feat: expand 5/2 lesson with pair activity, challenge question, and 15-question Kahoot
- Add "Be the Agent" pair activity (10 min, Teams-ready) with 9 age-tuned tasks
- Add open-ended challenge question to class activity (flight booking failure scenario)
- Expand Kahoot from 12 to 15 questions (hallucinations, "Act" step, memory vs tools)
- Standardize Kahoot at 15 questions for all future lessons in CLAUDE.md

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/2026-05-02_How_AI_Agents_Work/2026-05-02_Kahoot_Import.xlsx
+++ b/2026-05-02_How_AI_Agents_Work/2026-05-02_Kahoot_Import.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -849,6 +849,105 @@
         <v>2</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>What is an AI 'hallucination'?</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>When the AI sees pictures or images</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>When the AI confidently makes up an answer that isn't true</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>When the AI runs out of memory</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>When the AI uses too many tools at once</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>20</v>
+      </c>
+      <c r="G14" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>In the agent loop, what is the 'Act' step?</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>The agent talks back to the user</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>The agent uses a tool to do something (search, send email, run code)</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>The agent thinks about its options</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>The agent saves its memory</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>20</v>
+      </c>
+      <c r="G15" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>An assistant has MEMORY but no TOOLS. Which task can it still NOT do?</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Remember your name from earlier in the chat</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Look up today's weather</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Write a poem about your dog</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Answer trivia from its training data</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>25</v>
+      </c>
+      <c r="G16" t="n">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>